<commit_message>
Add remaining document template detection rules
</commit_message>
<xml_diff>
--- a/config/taxonomy_config_v5.xlsx
+++ b/config/taxonomy_config_v5.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -575,6 +575,402 @@
         <v>80</v>
       </c>
       <c r="H4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>laudo_mps</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Laudo analitico de material particulado em suspensao</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Template para laudos analiticos de MPS/material particulado.</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>15</v>
+      </c>
+      <c r="G5" t="n">
+        <v>80</v>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>template_laudo_ect_v1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>laudo_ect</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Laudo de ensaio ecotoxicologico</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Template para relatorios de analises/ensaios ecotoxicologicos Aplysia.</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>40</v>
+      </c>
+      <c r="G6" t="n">
+        <v>80</v>
+      </c>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>laudo_zbt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Laudo de zoobentos</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Template para relatorios de ensaio de macroinvertebrados bentonicos/zoobentos.</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>50</v>
+      </c>
+      <c r="G7" t="n">
+        <v>80</v>
+      </c>
+      <c r="H7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>template_laudo_dsl_v1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>laudo_dsl</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Laudo de descarga liquida</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Template para relatorios de ensaio de descarga liquida/vazao.</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>60</v>
+      </c>
+      <c r="G8" t="n">
+        <v>80</v>
+      </c>
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>template_laudo_dss_v1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>laudo_dss</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Laudo de descarga solida</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Template para relatorios de ensaio de descarga solida.</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>70</v>
+      </c>
+      <c r="G9" t="n">
+        <v>80</v>
+      </c>
+      <c r="H9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>template_ficha_coleta_tommasi_v1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ficha_coleta_tommasi</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Ficha de coleta / cadeia de custodia Tommasi</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Template para cadeias de custodia e fichas de coleta Tommasi.</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>80</v>
+      </c>
+      <c r="G10" t="n">
+        <v>80</v>
+      </c>
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_aplysia_v1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_aplysia</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Ficha de recebimento Aplysia</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Template para confirmacao/checklist de recebimento de amostras Aplysia.</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>90</v>
+      </c>
+      <c r="G11" t="n">
+        <v>80</v>
+      </c>
+      <c r="H11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_labmar_v1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_labmar</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ficha de recebimento Labmar</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Template para checklist de recebimento Labmar.</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>100</v>
+      </c>
+      <c r="G12" t="n">
+        <v>80</v>
+      </c>
+      <c r="H12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_ethica_v1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_ethica</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ficha de recebimento Ethica</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Template para checklist/planilha de recebimento Ethica.</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>110</v>
+      </c>
+      <c r="G13" t="n">
+        <v>80</v>
+      </c>
+      <c r="H13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>template_ficha_subcontratacao_als_v1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ficha_subcontratacao_als</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Ficha de subcontratacao ALS</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Template para fichas FO-ANL-098 de subcontratacao de servicos de analise ALS Corplab.</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>120</v>
+      </c>
+      <c r="G14" t="n">
+        <v>80</v>
+      </c>
+      <c r="H14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_bioagri_v1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_bioagri</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Ficha de recebimento Bioagri</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Template para checklists/fichas de recebimento de amostras Bioagri.</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>130</v>
+      </c>
+      <c r="G15" t="n">
+        <v>80</v>
+      </c>
+      <c r="H15" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3067,7 +3463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3962,6 +4358,2118 @@
       <c r="G27" t="inlineStr">
         <is>
           <t>Evita classificar laudo de sedimento como agua.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Relat.rio Anal.tico</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="b">
+        <v>1</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Estrutura basica de relatorio analitico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Resultados Anal.ticos</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="b">
+        <v>1</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Estrutura basica de relatorio analitico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Informa..es da Amostra</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="b">
+        <v>1</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Estrutura basica de relatorio analitico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>ID Amostra</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="b">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Estrutura basica de relatorio analitico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Material\s+Particulado</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>40</v>
+      </c>
+      <c r="F32" t="b">
+        <v>1</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Identifica amostra/material particulado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Carbono\s+Org.nico\s+Particulado|\bParticulado\b</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>30</v>
+      </c>
+      <c r="F33" t="b">
+        <v>1</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Parametros com particulado caracteristicos de MPS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>(?:\|/|_)MPS(?:\|/|_|\.)</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>30</v>
+      </c>
+      <c r="F34" t="b">
+        <v>1</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Caminho ou nome do arquivo indica MPS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Fitopl.ncton|Comunidade\s+Fitoplanct.nica|Macroinvertebrados|Zoobentos</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="b">
+        <v>1</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Evita confundir MPS com fito ou zoobentos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>template_laudo_ect_v1</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Relat.rio\s+de\s+an.lises</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="b">
+        <v>1</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Documento deve ser relatorio de analises.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>template_laudo_ect_v1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Ecotoxicologia\s+Aqu.tica|ensaios?\s+ecotoxicol.gicos?</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>40</v>
+      </c>
+      <c r="F37" t="b">
+        <v>1</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Tema ecotoxicologico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>template_laudo_ect_v1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>APLYSIA|Laborat.rio\s+de\s+Ecotoxicologia</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>30</v>
+      </c>
+      <c r="F38" t="b">
+        <v>1</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Laboratorio/formato Aplysia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>template_laudo_ect_v1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Ceriodaphnia|Daphnia|Hyalella|Raphidocelis|Vibrio\s+fischeri|Echinometra|Nitocra</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>30</v>
+      </c>
+      <c r="F39" t="b">
+        <v>1</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Organismos-teste caracteristicos de ECT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>template_laudo_ect_v1</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>(?:\|/|_)ECT(?:\|/|_|\.)|_ect_</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>20</v>
+      </c>
+      <c r="F40" t="b">
+        <v>1</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Caminho ou nome indica ECT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>template_laudo_ect_v1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Resultados\s+Anal.ticos|Relat.rio\s+Anal.tico\s+\d+</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="b">
+        <v>0</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Regra desativada: bloqueava relatorios de analises ECT validos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Relat.rio\s+de\s+Ensaio</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="b">
+        <v>0</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Documento deve ser relatorio de ensaio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Zoobentos|Macroinvertebrados\s+Bent.nicos|Macrofauna\s+de\s+fundo</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>45</v>
+      </c>
+      <c r="F43" t="b">
+        <v>1</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Tema de zoobentos/macrofauna bentonica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Ind\./m.|Fam.lia|Filo|Classe\s+\w+</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>25</v>
+      </c>
+      <c r="F44" t="b">
+        <v>1</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Resultados taxonomicos de bentos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>RESULTADOS|Identifica..o\s+do\s+Laborat.rio</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>20</v>
+      </c>
+      <c r="F45" t="b">
+        <v>1</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Secao de resultados do formato ZBT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>(?:\|/|_)ZBT(?:\|/|_|\.)|bentos</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>20</v>
+      </c>
+      <c r="F46" t="b">
+        <v>1</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Caminho ou nome indica ZBT/bentos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Descarga\s+L.quida|Descarga\s+S.lida|Ecotoxicologia</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="b">
+        <v>1</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Evita confundir com DSL/DSS/ECT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>template_laudo_dsl_v1</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>RELAT.RIO\s+DE\s+ENSAIO|Relat.rio\s+de\s+Ensaio</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="b">
+        <v>1</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Documento deve ser relatorio de ensaio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>template_laudo_dsl_v1</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Medi..o\s+de\s+Vaz.o|Descarga\s+L.quida</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>45</v>
+      </c>
+      <c r="F49" t="b">
+        <v>1</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Tema descarga liquida/vazao.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>template_laudo_dsl_v1</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ADCP|Tipo\s+de\s+medidor|Dados\s+do\s+equipamento</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>25</v>
+      </c>
+      <c r="F50" t="b">
+        <v>1</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Equipamento e metodologia de DSL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>template_laudo_dsl_v1</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Determina..o\s+da\s+descarga\s+l.quida</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>25</v>
+      </c>
+      <c r="F51" t="b">
+        <v>1</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Metodologia declarada de DSL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>template_laudo_dsl_v1</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>(?:\|/|_)DSL(?:\|/|_|\.)</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>20</v>
+      </c>
+      <c r="F52" t="b">
+        <v>1</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Caminho ou nome indica DSL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>template_laudo_dsl_v1</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Medi..o\s+de\s+Descarga\s+S.lida|Determina..o\s+da\s+descarga\s+s.lida|Einstein\s+Modificado|Colby\s+Simplificado</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="b">
+        <v>0</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Regra desativada: DSL pode mencionar planilhas de descarga solida no corpo do relatorio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>template_laudo_dss_v1</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>RELAT.RIO\s+DE\s+ENSAIO|Relat.rio\s+de\s+Ensaio</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="b">
+        <v>0</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Documento deve ser relatorio de ensaio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>template_laudo_dss_v1</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Medi..o\s+de\s+Descarga\s+S.lida|Descarga\s+S.lida</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>50</v>
+      </c>
+      <c r="F55" t="b">
+        <v>1</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Tema descarga solida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>template_laudo_dss_v1</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Einstein\s+Modificado|Colby\s+Simplificado</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>30</v>
+      </c>
+      <c r="F56" t="b">
+        <v>1</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Metodologias caracteristicas de DSS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>template_laudo_dss_v1</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Dados\s+de\s+Entrada|DADOS\s+D</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>15</v>
+      </c>
+      <c r="F57" t="b">
+        <v>1</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Secao de entrada caracteristica de DSS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>template_laudo_dss_v1</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>(?:\|/|_)DSS(?:\|/|_|\.)</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>20</v>
+      </c>
+      <c r="F58" t="b">
+        <v>1</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Caminho ou nome indica DSS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>template_laudo_dss_v1</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Descarga\s+L.quida|ADCP</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" t="b">
+        <v>0</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Regra desativada: DSS tambem pode citar descarga liquida/ADCP como dado de entrada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>template_ficha_coleta_tommasi_v1</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Cadeia\s+de\s+Cust.dia</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="b">
+        <v>1</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Documento deve ser cadeia de custodia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>template_ficha_coleta_tommasi_v1</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Amostra\s+Id|Identifica..o\s+ou\s+Ponto\s+de\s+Coleta</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>40</v>
+      </c>
+      <c r="F61" t="b">
+        <v>1</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Campos caracteristicos da ficha de coleta Tommasi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>template_ficha_coleta_tommasi_v1</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Embalagem\s+e\s+Preserva..o|Planejamento\s+de\s+Amostragem</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>30</v>
+      </c>
+      <c r="F62" t="b">
+        <v>1</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Campos de embalagem/planejamento de coleta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>template_ficha_coleta_tommasi_v1</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Checklist\s+de\s+recebimento|Data\s+e\s+Hora\s+de\s+Recebimento</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>20</v>
+      </c>
+      <c r="F63" t="b">
+        <v>1</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Checklist de recebimento acoplado a COC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>template_ficha_coleta_tommasi_v1</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Fichas\s+de\s+coleta</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>20</v>
+      </c>
+      <c r="F64" t="b">
+        <v>1</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Caminho indica ficha de coleta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>template_ficha_coleta_tommasi_v1</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Relat.rio\s+Anal.tico|Relat.rio\s+de\s+Ensaio|Confirma..o\s+de\s+Recebimento</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="b">
+        <v>1</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Evita confundir ficha com laudos ou recebimentos subcontratados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_aplysia_v1</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Confirma..o\s+de\s+Recebimento\s+de\s+Amostras</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="b">
+        <v>1</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Documento de confirmacao de recebimento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_aplysia_v1</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>APLYSIA</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>40</v>
+      </c>
+      <c r="F67" t="b">
+        <v>1</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Laboratorio Aplysia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_aplysia_v1</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Ensaios?\s+Ecotoxicol.gicos?|Daphnia|Ceriodaphnia|Hyalella|Raphidocelis</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>40</v>
+      </c>
+      <c r="F68" t="b">
+        <v>1</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Ensaios/organismos de ecotoxicologia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_aplysia_v1</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Aplysia</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>20</v>
+      </c>
+      <c r="F69" t="b">
+        <v>1</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Caminho indica Aplysia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_labmar_v1</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Checklist\s+de\s+Recebimento</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="b">
+        <v>1</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Documento checklist de recebimento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_labmar_v1</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>LABMAR|FM-LAB-035|LAUDO\s+VINCULADO</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>50</v>
+      </c>
+      <c r="F71" t="b">
+        <v>1</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Formato Labmar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_labmar_v1</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>N.?\s*PROPOSTA\s+COMERCIAL|DATA\s+DO\s+RECEBIMENTO</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>20</v>
+      </c>
+      <c r="F72" t="b">
+        <v>1</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Campos caracteristicos de recebimento Labmar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_labmar_v1</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Labmar</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>20</v>
+      </c>
+      <c r="F73" t="b">
+        <v>1</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Caminho indica Labmar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_ethica_v1</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>RESPONS.VEL\s+PELA\s+ENTREGA|RESPONS.VEL\s+PELO\s+RECEBIMENTO</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" t="b">
+        <v>0</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Regra desativada: alguns checklists Ethica nao possuem texto extraivel; caminho forte assume a identificacao.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_ethica_v1</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>ID\s+Amostra\s+Data\s*/\s*Hora\s+Coleta|Proposta\s+.*Comercial</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>40</v>
+      </c>
+      <c r="F75" t="b">
+        <v>1</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Cabecalho tabular Ethica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_ethica_v1</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Clorofila\s+e\s+Feofitina|Preservante|Refrigerado</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>30</v>
+      </c>
+      <c r="F76" t="b">
+        <v>1</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Campos/analises caracteristicas do recebimento Ethica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_ethica_v1</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>.thica|Ethica</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>20</v>
+      </c>
+      <c r="F77" t="b">
+        <v>1</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Caminho indica Ethica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Meiofauna\s+Bent.nica|Meiofauna\s+de\s+fundo</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>45</v>
+      </c>
+      <c r="F78" t="b">
+        <v>1</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Reconhece laudos ZBT de meiofauna bentonica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>(?:\|/|_)Sed(?:\|/|_|\.)</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>40</v>
+      </c>
+      <c r="F79" t="b">
+        <v>1</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Caminho ou nome indica laudo de sedimento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Sedimento\s*-\s*Branco\s+de\s+equipamento|Sedimento\s*-\s*Branco</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>40</v>
+      </c>
+      <c r="F80" t="b">
+        <v>1</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Reconhece branco de equipamento associado a sedimento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>template_ficha_subcontratacao_als_v1</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>SUBCONTRATA..O\s+DE\s+SERVI.OS\s+DE\s+AN.LISE|FO-ANL-098</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" t="b">
+        <v>1</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Documento de subcontratacao de servicos de analise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>template_ficha_subcontratacao_als_v1</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Provedor\s+Externo:\s*ALS|ALS\s+Corplab</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>50</v>
+      </c>
+      <c r="F82" t="b">
+        <v>1</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Provedor externo ALS Corplab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>template_ficha_subcontratacao_als_v1</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>ID\s+Amostra\s+Identifica..o\s+Data/Hora\s+Coleta|Matriz\s+An.lise\s+Metodologia</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>30</v>
+      </c>
+      <c r="F83" t="b">
+        <v>1</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Cabecalho tabular da ficha ALS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>template_ficha_subcontratacao_als_v1</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>COC_subcontratadas.*ALS|ALS</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>30</v>
+      </c>
+      <c r="F84" t="b">
+        <v>1</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Caminho indica subcontratada ALS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>template_ficha_subcontratacao_als_v1</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Relat.rio\s+Anal.tico|Relat.rio\s+de\s+Ensaio|Cadeia\s+de\s+Cust.dia</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" t="b">
+        <v>1</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Evita confundir ficha ALS com laudos ou COC principal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_bioagri_v1</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>COC_subcontratadas.*Bioagri|Bioagri</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>85</v>
+      </c>
+      <c r="F86" t="b">
+        <v>1</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Caminho indica recebimento/checklist Bioagri.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_bioagri_v1</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Checklist\s+de\s+Recebimento</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>20</v>
+      </c>
+      <c r="F87" t="b">
+        <v>1</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Nome do arquivo indica checklist de recebimento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_bioagri_v1</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Relat.rio\s+Anal.tico|Relat.rio\s+de\s+Ensaio|Cadeia\s+de\s+Cust.dia</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" t="b">
+        <v>1</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Evita confundir checklist Bioagri com laudos ou COC principal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_ethica_v1</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>COC_subcontratadas.*(?:.thica|Ethica)</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>85</v>
+      </c>
+      <c r="F89" t="b">
+        <v>1</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Caminho forte indica recebimento Ethica em subcontratadas, inclusive em PDF sem texto extraivel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>\\ZBT\\|/ZBT/|_bentos\.pdf|bentos</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>90</v>
+      </c>
+      <c r="F90" t="b">
+        <v>1</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Caminho ou nome indica laudo ZBT/bentos quando o PDF nao tem texto extraivel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>template_laudo_dss_v1</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>\\DSS\\|/DSS/</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>90</v>
+      </c>
+      <c r="F91" t="b">
+        <v>1</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Caminho indica laudo DSS quando o PDF nao tem texto extraivel.</t>
         </is>
       </c>
     </row>
@@ -3976,7 +6484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4426,6 +6934,1546 @@
         <v>1</v>
       </c>
       <c r="F16" t="inlineStr">
+        <is>
+          <t>Erros de validacao da saida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>laudo_mps</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Resultados extraidos do PDF para o template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>laudo_mps</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="b">
+        <v>1</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Dados de amostra/cabecalho do PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>laudo_mps</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>laudo_mps</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>98</v>
+      </c>
+      <c r="E20" t="b">
+        <v>1</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>laudo_mps</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>validation_errors</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>99</v>
+      </c>
+      <c r="E21" t="b">
+        <v>1</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Erros de validacao da saida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>template_laudo_ect_v1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>laudo_ect</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="b">
+        <v>1</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Resultados extraidos do PDF para o template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>template_laudo_ect_v1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>laudo_ect</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" t="b">
+        <v>1</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Dados de amostra/cabecalho do PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>template_laudo_ect_v1</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>laudo_ect</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" t="b">
+        <v>1</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>template_laudo_ect_v1</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>laudo_ect</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>98</v>
+      </c>
+      <c r="E25" t="b">
+        <v>1</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>template_laudo_ect_v1</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>laudo_ect</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>validation_errors</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>99</v>
+      </c>
+      <c r="E26" t="b">
+        <v>1</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Erros de validacao da saida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>laudo_zbt</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="b">
+        <v>1</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Resultados extraidos do PDF para o template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>laudo_zbt</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" t="b">
+        <v>1</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Dados de amostra/cabecalho do PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>laudo_zbt</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" t="b">
+        <v>1</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>laudo_zbt</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>98</v>
+      </c>
+      <c r="E30" t="b">
+        <v>1</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>laudo_zbt</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>validation_errors</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>99</v>
+      </c>
+      <c r="E31" t="b">
+        <v>1</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Erros de validacao da saida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>template_laudo_dsl_v1</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>laudo_dsl</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="b">
+        <v>1</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Resultados extraidos do PDF para o template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>template_laudo_dsl_v1</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>laudo_dsl</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E33" t="b">
+        <v>1</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Dados de amostra/cabecalho do PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>template_laudo_dsl_v1</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>laudo_dsl</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" t="b">
+        <v>1</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>template_laudo_dsl_v1</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>laudo_dsl</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>98</v>
+      </c>
+      <c r="E35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>template_laudo_dsl_v1</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>laudo_dsl</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>validation_errors</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>99</v>
+      </c>
+      <c r="E36" t="b">
+        <v>1</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Erros de validacao da saida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>template_laudo_dss_v1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>laudo_dss</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="b">
+        <v>1</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Resultados extraidos do PDF para o template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>template_laudo_dss_v1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>laudo_dss</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>2</v>
+      </c>
+      <c r="E38" t="b">
+        <v>1</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Dados de amostra/cabecalho do PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>template_laudo_dss_v1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>laudo_dss</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" t="b">
+        <v>1</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>template_laudo_dss_v1</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>laudo_dss</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>98</v>
+      </c>
+      <c r="E40" t="b">
+        <v>1</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>template_laudo_dss_v1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>laudo_dss</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>validation_errors</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>99</v>
+      </c>
+      <c r="E41" t="b">
+        <v>1</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Erros de validacao da saida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>template_ficha_coleta_tommasi_v1</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ficha_coleta_tommasi</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="b">
+        <v>1</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Resultados extraidos do PDF para o template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>template_ficha_coleta_tommasi_v1</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ficha_coleta_tommasi</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" t="b">
+        <v>1</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Dados de amostra/cabecalho do PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>template_ficha_coleta_tommasi_v1</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ficha_coleta_tommasi</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" t="b">
+        <v>1</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>template_ficha_coleta_tommasi_v1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ficha_coleta_tommasi</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>98</v>
+      </c>
+      <c r="E45" t="b">
+        <v>1</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>template_ficha_coleta_tommasi_v1</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ficha_coleta_tommasi</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>validation_errors</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>99</v>
+      </c>
+      <c r="E46" t="b">
+        <v>1</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Erros de validacao da saida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_aplysia_v1</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_aplysia</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" t="b">
+        <v>1</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Resultados extraidos do PDF para o template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_aplysia_v1</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_aplysia</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>2</v>
+      </c>
+      <c r="E48" t="b">
+        <v>1</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Dados de amostra/cabecalho do PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_aplysia_v1</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_aplysia</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" t="b">
+        <v>1</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_aplysia_v1</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_aplysia</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>98</v>
+      </c>
+      <c r="E50" t="b">
+        <v>1</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_aplysia_v1</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_aplysia</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>validation_errors</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>99</v>
+      </c>
+      <c r="E51" t="b">
+        <v>1</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Erros de validacao da saida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_labmar_v1</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_labmar</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" t="b">
+        <v>1</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Resultados extraidos do PDF para o template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_labmar_v1</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_labmar</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>2</v>
+      </c>
+      <c r="E53" t="b">
+        <v>1</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Dados de amostra/cabecalho do PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_labmar_v1</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_labmar</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>3</v>
+      </c>
+      <c r="E54" t="b">
+        <v>1</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_labmar_v1</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_labmar</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>98</v>
+      </c>
+      <c r="E55" t="b">
+        <v>1</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_labmar_v1</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_labmar</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>validation_errors</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>99</v>
+      </c>
+      <c r="E56" t="b">
+        <v>1</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Erros de validacao da saida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_ethica_v1</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_ethica</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" t="b">
+        <v>1</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Resultados extraidos do PDF para o template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_ethica_v1</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_ethica</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" t="b">
+        <v>1</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Dados de amostra/cabecalho do PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_ethica_v1</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_ethica</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>3</v>
+      </c>
+      <c r="E59" t="b">
+        <v>1</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_ethica_v1</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_ethica</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>98</v>
+      </c>
+      <c r="E60" t="b">
+        <v>1</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_ethica_v1</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_ethica</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>validation_errors</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>99</v>
+      </c>
+      <c r="E61" t="b">
+        <v>1</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Erros de validacao da saida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>template_ficha_subcontratacao_als_v1</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>ficha_subcontratacao_als</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" t="b">
+        <v>1</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Resultados extraidos do PDF para o template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>template_ficha_subcontratacao_als_v1</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>ficha_subcontratacao_als</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>2</v>
+      </c>
+      <c r="E63" t="b">
+        <v>1</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Dados de amostra/cabecalho do PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>template_ficha_subcontratacao_als_v1</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>ficha_subcontratacao_als</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>3</v>
+      </c>
+      <c r="E64" t="b">
+        <v>1</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>template_ficha_subcontratacao_als_v1</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>ficha_subcontratacao_als</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>98</v>
+      </c>
+      <c r="E65" t="b">
+        <v>1</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>template_ficha_subcontratacao_als_v1</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>ficha_subcontratacao_als</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>validation_errors</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>99</v>
+      </c>
+      <c r="E66" t="b">
+        <v>1</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Erros de validacao da saida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_bioagri_v1</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_bioagri</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" t="b">
+        <v>1</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Resultados extraidos do PDF para o template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_bioagri_v1</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_bioagri</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>2</v>
+      </c>
+      <c r="E68" t="b">
+        <v>1</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Dados de amostra/cabecalho do PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_bioagri_v1</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_bioagri</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>3</v>
+      </c>
+      <c r="E69" t="b">
+        <v>1</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_bioagri_v1</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_bioagri</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>98</v>
+      </c>
+      <c r="E70" t="b">
+        <v>1</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>template_ficha_recebimento_bioagri_v1</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ficha_recebimento_bioagri</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>validation_errors</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>99</v>
+      </c>
+      <c r="E71" t="b">
+        <v>1</v>
+      </c>
+      <c r="F71" t="inlineStr">
         <is>
           <t>Erros de validacao da saida.</t>
         </is>
@@ -6283,6 +10331,7 @@
           <t>Amostragem</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>campo</t>
@@ -6308,6 +10357,7 @@
           <t>Físico-Químico</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>laboratorio</t>
@@ -6333,6 +10383,7 @@
           <t>Constituintes inorgânicos não metálicos</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>laboratorio</t>
@@ -6358,6 +10409,7 @@
           <t>Constituintes orgânicos agregados</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>laboratorio</t>
@@ -6383,6 +10435,7 @@
           <t>Metais</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>laboratorio</t>
@@ -6408,6 +10461,7 @@
           <t>Microbiológicos</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>laboratorio</t>
@@ -6433,6 +10487,7 @@
           <t>Propriedades físicas e agregadas</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>laboratorio</t>
@@ -6458,6 +10513,7 @@
           <t>Ethica Ambiental</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>laboratorio</t>
@@ -6483,6 +10539,7 @@
           <t>Constituintes org?nicos agregados</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>laboratorio</t>
@@ -6508,6 +10565,7 @@
           <t>Constituintes org?nicos agregados</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>laboratorio</t>
@@ -6627,6 +10685,7 @@
       <c r="C2" t="n">
         <v>1</v>
       </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
         <v>2</v>
       </c>
@@ -6642,6 +10701,12 @@
       <c r="I2" t="n">
         <v>6</v>
       </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="b">
         <v>1</v>
       </c>
@@ -6663,12 +10728,21 @@
       <c r="D3" t="n">
         <v>3</v>
       </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
         <v>4</v>
       </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
         <v>1</v>
       </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="b">
         <v>1</v>
       </c>
@@ -6690,6 +10764,11 @@
       <c r="D4" t="n">
         <v>4</v>
       </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="n">
         <v>1</v>
       </c>
@@ -6702,6 +10781,8 @@
       <c r="M4" t="n">
         <v>6</v>
       </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
       <c r="P4" t="b">
         <v>1</v>
       </c>
@@ -6723,12 +10804,19 @@
       <c r="D5" t="n">
         <v>3</v>
       </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
         <v>1</v>
       </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>4</v>
       </c>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Replicate header schemas for fito and sediment templates
</commit_message>
<xml_diff>
--- a/config/taxonomy_config_v5.xlsx
+++ b/config/taxonomy_config_v5.xlsx
@@ -9675,7 +9675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9797,6 +9797,206 @@
         </is>
       </c>
       <c r="D6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>id_amostra</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ID Amostra:\s*(\d+)</t>
+        </is>
+      </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>latitude</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Latitude:\s*([-\d,]+)</t>
+        </is>
+      </c>
+      <c r="D8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>longitude</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Longitude:\s*([-\d,]+)</t>
+        </is>
+      </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>data_coleta</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Data Coleta:\s*(\d{2}/\d{2}/\d{4})</t>
+        </is>
+      </c>
+      <c r="D10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>subtipo_amostra</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Relatório Analítico\s*\d+/\d+\.\d+\.?([A-Z]{1,2})?</t>
+        </is>
+      </c>
+      <c r="D11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>id_amostra</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ID Amostra:\s*(\d+)</t>
+        </is>
+      </c>
+      <c r="D12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>latitude</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Latitude:\s*([-\d,]+)</t>
+        </is>
+      </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>longitude</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Longitude:\s*([-\d,]+)</t>
+        </is>
+      </c>
+      <c r="D14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>data_coleta</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Data Coleta:\s*(\d{2}/\d{2}/\d{4})</t>
+        </is>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>subtipo_amostra</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Relatório Analítico\s*\d+/\d+\.\d+\.?([A-Z]{1,2})?</t>
+        </is>
+      </c>
+      <c r="D16" t="b">
         <v>1</v>
       </c>
     </row>
@@ -9811,7 +10011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10013,6 +10213,356 @@
         </is>
       </c>
       <c r="E8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>nome_do_arquivo</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DERIVADO_DO_NOME_DO_PDF</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Nome do arquivo PDF de origem da extracao.</t>
+        </is>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>proposta_comercial</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Proposta Comercial:\s*(.*?)(?:\n|\s+Identifica..o do Cliente)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Codigo da proposta comercial informado no cabecalho.</t>
+        </is>
+      </c>
+      <c r="E10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>cliente</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Cliente:\s*(.*?)(?:\s+CNPJ/CPF:|\n)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Nome do cliente.</t>
+        </is>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>cnpj_cpf</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CNPJ/CPF:\s*([\d./-]+)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Documento do cliente.</t>
+        </is>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>contato</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Contato:\s*(.*?)(?:\s+Telefone:|\n)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Contato do cliente.</t>
+        </is>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>telefone</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Telefone:\s*([\d\s()+-]+)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Telefone do contato do cliente.</t>
+        </is>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>endereco</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Endere..o:\s*(.*?)(?:\nInforma..es da Amostra|\n)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Endereco do cliente, quando informado.</t>
+        </is>
+      </c>
+      <c r="E15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nome_do_arquivo</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>DERIVADO_DO_NOME_DO_PDF</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Nome do arquivo PDF de origem da extracao.</t>
+        </is>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>proposta_comercial</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Proposta Comercial:\s*(.*?)(?:\n|\s+Identifica..o do Cliente)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Codigo da proposta comercial informado no cabecalho.</t>
+        </is>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>cliente</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Cliente:\s*(.*?)(?:\s+CNPJ/CPF:|\n)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Nome do cliente.</t>
+        </is>
+      </c>
+      <c r="E18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>cnpj_cpf</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CNPJ/CPF:\s*([\d./-]+)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Documento do cliente.</t>
+        </is>
+      </c>
+      <c r="E19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>contato</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Contato:\s*(.*?)(?:\s+Telefone:|\n)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Contato do cliente.</t>
+        </is>
+      </c>
+      <c r="E20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>telefone</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Telefone:\s*([\d\s()+-]+)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Telefone do contato do cliente.</t>
+        </is>
+      </c>
+      <c r="E21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>endereco</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Endere..o:\s*(.*?)(?:\nInforma..es da Amostra|\n)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Endereco do cliente, quando informado.</t>
+        </is>
+      </c>
+      <c r="E22" t="b">
         <v>1</v>
       </c>
     </row>
@@ -10027,7 +10577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10369,6 +10919,646 @@
         </is>
       </c>
       <c r="D17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nome_do_arquivo</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>DERIVADO_DO_NOME_DO_PDF</t>
+        </is>
+      </c>
+      <c r="D18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>tipo_amostra</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Tipo de Amostra:\s*(.*?)(?:\s+ID Amostra:|\n)</t>
+        </is>
+      </c>
+      <c r="D19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>criterio_conformidade</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Crit.rio de Conformidade:\s*(.*?)(?:\s+Data Coleta:|\n)</t>
+        </is>
+      </c>
+      <c r="D20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>dh_coleta</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Data Coleta:\s*\d{2}/\d{2}/\d{4}\s+(\d{2}:\d{2})</t>
+        </is>
+      </c>
+      <c r="D21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>data_publicacao</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Data de Publica..o:\s*(\d{2}/\d{2}/\d{4})</t>
+        </is>
+      </c>
+      <c r="D22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>dh_publicacao</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Data de Publica..o:\s*\d{2}/\d{2}/\d{4}\s+(\d{2}:\d{2})</t>
+        </is>
+      </c>
+      <c r="D23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>data_recebimento</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Data de Recebimento:\s*(\d{2}/\d{2}/\d{4})</t>
+        </is>
+      </c>
+      <c r="D24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>dh_recebimento</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Data de Recebimento:\s*\d{2}/\d{2}/\d{4}\s+(\d{2}:\d{2})</t>
+        </is>
+      </c>
+      <c r="D25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>observacoes</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Observa..es:\s*(.*?)(?:\s+Latitude:|\n)</t>
+        </is>
+      </c>
+      <c r="D26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>clima_ultimas_24h</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Condi..es clim.ticas nas .ltimas 24 horas:\s*(.*?)(?:\s+Condi..es clim.ticas no momento da coleta:|\n)</t>
+        </is>
+      </c>
+      <c r="D27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>clima</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Condi..es clim.ticas no momento da coleta:\s*(.*?)(?:\s+Local da Coleta:|\n)</t>
+        </is>
+      </c>
+      <c r="D28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>localizacao</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Local da Coleta:\s*(.*?)(?:\s+Tipo de Coleta:|\n)</t>
+        </is>
+      </c>
+      <c r="D29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>tipo_coleta</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Tipo de Coleta:\s*(.*?)(?:\s+Responsabilidade da Amostragem:|\n)</t>
+        </is>
+      </c>
+      <c r="D30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>responsavel_amostra</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Responsabilidade da Amostragem:\s*(.*?)(?:\s+Descri..o|\s+Planejamento|\n)</t>
+        </is>
+      </c>
+      <c r="D31" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>planejamento_amostragem</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Planejamento de Amostragem:\s*(.*?)(?:\s+conformidade|\n)</t>
+        </is>
+      </c>
+      <c r="D32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>template_laudo_fito_v1</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>descricao_nao_conformidade</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Descri..o da n.o-conformidade:\s*(.*?)(?:\s+Planejamento de Amostragem:|\n)</t>
+        </is>
+      </c>
+      <c r="D33" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>nome_do_arquivo</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>DERIVADO_DO_NOME_DO_PDF</t>
+        </is>
+      </c>
+      <c r="D34" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>tipo_amostra</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Tipo de Amostra:\s*(.*?)(?:\s+ID Amostra:|\n)</t>
+        </is>
+      </c>
+      <c r="D35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>criterio_conformidade</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Crit.rio de Conformidade:\s*(.*?)(?:\s+Data Coleta:|\n)</t>
+        </is>
+      </c>
+      <c r="D36" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>dh_coleta</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Data Coleta:\s*\d{2}/\d{2}/\d{4}\s+(\d{2}:\d{2})</t>
+        </is>
+      </c>
+      <c r="D37" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>data_publicacao</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Data de Publica..o:\s*(\d{2}/\d{2}/\d{4})</t>
+        </is>
+      </c>
+      <c r="D38" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>dh_publicacao</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Data de Publica..o:\s*\d{2}/\d{2}/\d{4}\s+(\d{2}:\d{2})</t>
+        </is>
+      </c>
+      <c r="D39" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>data_recebimento</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Data de Recebimento:\s*(\d{2}/\d{2}/\d{4})</t>
+        </is>
+      </c>
+      <c r="D40" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>dh_recebimento</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Data de Recebimento:\s*\d{2}/\d{2}/\d{4}\s+(\d{2}:\d{2})</t>
+        </is>
+      </c>
+      <c r="D41" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>observacoes</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Observa..es:\s*(.*?)(?:\s+Latitude:|\n)</t>
+        </is>
+      </c>
+      <c r="D42" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>clima_ultimas_24h</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Condi..es clim.ticas nas .ltimas 24 horas:\s*(.*?)(?:\s+Condi..es clim.ticas no momento da coleta:|\n)</t>
+        </is>
+      </c>
+      <c r="D43" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>clima</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Condi..es clim.ticas no momento da coleta:\s*(.*?)(?:\s+Local da Coleta:|\n)</t>
+        </is>
+      </c>
+      <c r="D44" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>localizacao</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Local da Coleta:\s*(.*?)(?:\s+Tipo de Coleta:|\n)</t>
+        </is>
+      </c>
+      <c r="D45" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>tipo_coleta</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Tipo de Coleta:\s*(.*?)(?:\s+Responsabilidade da Amostragem:|\n)</t>
+        </is>
+      </c>
+      <c r="D46" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>responsavel_amostra</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Responsabilidade da Amostragem:\s*(.*?)(?:\s+Descri..o|\s+Planejamento|\n)</t>
+        </is>
+      </c>
+      <c r="D47" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>planejamento_amostragem</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Planejamento de Amostragem:\s*(.*?)(?:\s+conformidade|\n)</t>
+        </is>
+      </c>
+      <c r="D48" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>descricao_nao_conformidade</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Descri..o da n.o-conformidade:\s*(.*?)(?:\s+Planejamento de Amostragem:|\n)</t>
+        </is>
+      </c>
+      <c r="D49" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Use only PDF text for taxonomy detection
</commit_message>
<xml_diff>
--- a/config/taxonomy_config_v5.xlsx
+++ b/config/taxonomy_config_v5.xlsx
@@ -3599,7 +3599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -3675,7 +3675,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>laudo</t>
+          <t>ficha_campo</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3685,30 +3685,30 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>path</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Laudos?|relat.rio</t>
+          <t>Ficha\s+de\s+Campo|Dados\s+de\s+Campo|Medi..o\s+em\s+Campo</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Caminho indica pasta de laudos.</t>
+          <t>Estrutura textual comum de ficha de campo.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ficha_campo</t>
+          <t>ficha_coleta</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3723,25 +3723,25 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ficha\s+de\s+Campo|Dados\s+de\s+Campo|Medi..o\s+em\s+Campo</t>
+          <t>Cadeia\s+de\s+Cust.dia\s*:|Amostra\s+Id\s*:|Identifica..o\s+ou\s+Ponto\s+de\s+Coleta\s*:</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Estrutura textual comum de ficha de campo.</t>
+          <t>Campos textuais especificos de ficha de coleta/cadeia de custodia.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ficha_campo</t>
+          <t>ficha_recebimento</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3751,30 +3751,30 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>filename</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>campo</t>
+          <t>Confirma..o\s+de\s+Recebimento|Checklist\s+de\s+Recebimento|RECEBIMENTO\s+DE\s+AMOSTRAS|RESPONS.VEL\s+PELA\s+ENTREGA</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Nome do arquivo indica campo.</t>
+          <t>Estrutura textual comum de ficha de recebimento.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ficha_coleta</t>
+          <t>ficha_subcontratacao</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3789,216 +3789,18 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Cadeia\s+de\s+Cust.dia|Planejamento\s+de\s+Amostragem|Amostra\s+Id</t>
+          <t>SUBCONTRATA..O\s+DE\s+SERVI.OS\s+DE\s+AN.LISE|Provedor\s+Externo</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Estrutura textual comum de ficha de coleta/cadeia de custodia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>ficha_coleta</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>path</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Fichas?\s+de\s+coleta|coleta</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>30</v>
-      </c>
-      <c r="F7" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Caminho indica ficha de coleta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ficha_recebimento</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Confirma..o\s+de\s+Recebimento|Checklist\s+de\s+Recebimento|RESPONS.VEL\s+PELA\s+ENTREGA</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>70</v>
-      </c>
-      <c r="F8" t="b">
-        <v>1</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Estrutura textual comum de ficha de recebimento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>ficha_recebimento</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>filename</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>recebimento|checklist</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>30</v>
-      </c>
-      <c r="F9" t="b">
-        <v>1</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Nome do arquivo indica recebimento/checklist.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ficha_recebimento</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>path</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>COC_subcontratadas|recebimento</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>20</v>
-      </c>
-      <c r="F10" t="b">
-        <v>1</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Caminho indica recebimento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>ficha_subcontratacao</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>SUBCONTRATA..O\s+DE\s+SERVI.OS\s+DE\s+AN.LISE|Provedor\s+Externo</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>70</v>
-      </c>
-      <c r="F11" t="b">
-        <v>1</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
           <t>Estrutura textual comum de subcontratacao.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>ficha_subcontratacao</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>path</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>COC_subcontratadas|subcontratad</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>30</v>
-      </c>
-      <c r="F12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Caminho indica subcontratacao.</t>
         </is>
       </c>
     </row>
@@ -4648,7 +4450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5700,7 +5502,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F32" t="b">
         <v>1</v>
@@ -5752,40 +5554,40 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>path</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>(?:\|/|_)MPS(?:\|/|_|\.)</t>
+          <t>Fitopl.ncton|Comunidade\s+Fitoplanct.nica|Macroinvertebrados|Zoobentos</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F34" t="b">
         <v>1</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Caminho ou nome do arquivo indica MPS.</t>
+          <t>Evita confundir MPS com fito ou zoobentos.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>template_laudo_mps_v1</t>
+          <t>template_laudo_ect_v1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>required</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -5795,7 +5597,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Fitopl.ncton|Comunidade\s+Fitoplanct.nica|Macroinvertebrados|Zoobentos</t>
+          <t>Relat.rio\s+de\s+an.lises</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -5806,7 +5608,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Evita confundir MPS com fito ou zoobentos.</t>
+          <t>Documento deve ser relatorio de analises.</t>
         </is>
       </c>
     </row>
@@ -5818,7 +5620,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>required</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5828,18 +5630,18 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Relat.rio\s+de\s+an.lises</t>
+          <t>Ecotoxicologia\s+Aqu.tica|ensaios?\s+ecotoxicol.gicos?</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F36" t="b">
         <v>1</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Documento deve ser relatorio de analises.</t>
+          <t>Tema ecotoxicologico.</t>
         </is>
       </c>
     </row>
@@ -5861,18 +5663,18 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Ecotoxicologia\s+Aqu.tica|ensaios?\s+ecotoxicol.gicos?</t>
+          <t>APLYSIA|Laborat.rio\s+de\s+Ecotoxicologia</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F37" t="b">
         <v>1</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Tema ecotoxicologico.</t>
+          <t>Laboratorio/formato Aplysia.</t>
         </is>
       </c>
     </row>
@@ -5894,7 +5696,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>APLYSIA|Laborat.rio\s+de\s+Ecotoxicologia</t>
+          <t>Ceriodaphnia|Daphnia|Hyalella|Raphidocelis|Vibrio\s+fischeri|Echinometra|Nitocra</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -5905,7 +5707,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Laboratorio/formato Aplysia.</t>
+          <t>Organismos-teste caracteristicos de ECT.</t>
         </is>
       </c>
     </row>
@@ -5917,7 +5719,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -5927,63 +5729,63 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Ceriodaphnia|Daphnia|Hyalella|Raphidocelis|Vibrio\s+fischeri|Echinometra|Nitocra</t>
+          <t>Resultados\s+Anal.ticos|Relat.rio\s+Anal.tico\s+\d+</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Organismos-teste caracteristicos de ECT.</t>
+          <t>Regra desativada: bloqueava relatorios de analises ECT validos.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>template_laudo_ect_v1</t>
+          <t>template_laudo_zbt_v1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>required</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>path</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>(?:\|/|_)ECT(?:\|/|_|\.)|_ect_</t>
+          <t>Relat.rio\s+de\s+Ensaio</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Caminho ou nome indica ECT.</t>
+          <t>Documento deve ser relatorio de ensaio.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>template_laudo_ect_v1</t>
+          <t>template_laudo_zbt_v1</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -5993,18 +5795,18 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Resultados\s+Anal.ticos|Relat.rio\s+Anal.tico\s+\d+</t>
+          <t>Zoobentos|Macroinvertebrados\s+Bent.nicos|Macrofauna\s+de\s+fundo</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Regra desativada: bloqueava relatorios de analises ECT validos.</t>
+          <t>Tema de zoobentos/macrofauna bentonica.</t>
         </is>
       </c>
     </row>
@@ -6016,7 +5818,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>required</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -6026,18 +5828,18 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Relat.rio\s+de\s+Ensaio</t>
+          <t>Ind\./m.|Fam.lia|Filo|Classe\s+\w+</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Documento deve ser relatorio de ensaio.</t>
+          <t>Resultados taxonomicos de bentos.</t>
         </is>
       </c>
     </row>
@@ -6059,18 +5861,18 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Zoobentos|Macroinvertebrados\s+Bent.nicos|Macrofauna\s+de\s+fundo</t>
+          <t>RESULTADOS|Identifica..o\s+do\s+Laborat.rio</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="F43" t="b">
         <v>1</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Tema de zoobentos/macrofauna bentonica.</t>
+          <t>Secao de resultados do formato ZBT.</t>
         </is>
       </c>
     </row>
@@ -6082,7 +5884,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -6092,30 +5894,30 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Ind\./m.|Fam.lia|Filo|Classe\s+\w+</t>
+          <t>Descarga\s+L.quida|Descarga\s+S.lida|Ecotoxicologia</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F44" t="b">
         <v>1</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Resultados taxonomicos de bentos.</t>
+          <t>Evita confundir com DSL/DSS/ECT.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>template_laudo_zbt_v1</t>
+          <t>template_laudo_dsl_v1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>required</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -6125,25 +5927,25 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>RESULTADOS|Identifica..o\s+do\s+Laborat.rio</t>
+          <t>RELAT.RIO\s+DE\s+ENSAIO|Relat.rio\s+de\s+Ensaio</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F45" t="b">
         <v>1</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Secao de resultados do formato ZBT.</t>
+          <t>Documento deve ser relatorio de ensaio.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>template_laudo_zbt_v1</t>
+          <t>template_laudo_dsl_v1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -6153,35 +5955,35 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>path</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>(?:\|/|_)ZBT(?:\|/|_|\.)|bentos</t>
+          <t>Medi..o\s+de\s+Vaz.o|Descarga\s+L.quida</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="F46" t="b">
         <v>1</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Caminho ou nome indica ZBT/bentos.</t>
+          <t>Tema descarga liquida/vazao.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>template_laudo_zbt_v1</t>
+          <t>template_laudo_dsl_v1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -6191,18 +5993,18 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Descarga\s+L.quida|Descarga\s+S.lida|Ecotoxicologia</t>
+          <t>ADCP|Tipo\s+de\s+medidor|Dados\s+do\s+equipamento</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F47" t="b">
         <v>1</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Evita confundir com DSL/DSS/ECT.</t>
+          <t>Equipamento e metodologia de DSL.</t>
         </is>
       </c>
     </row>
@@ -6214,7 +6016,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>required</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -6224,18 +6026,18 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>RELAT.RIO\s+DE\s+ENSAIO|Relat.rio\s+de\s+Ensaio</t>
+          <t>Determina..o\s+da\s+descarga\s+l.quida</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F48" t="b">
         <v>1</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Documento deve ser relatorio de ensaio.</t>
+          <t>Metodologia declarada de DSL.</t>
         </is>
       </c>
     </row>
@@ -6247,7 +6049,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -6257,30 +6059,30 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Medi..o\s+de\s+Vaz.o|Descarga\s+L.quida</t>
+          <t>Medi..o\s+de\s+Descarga\s+S.lida|Determina..o\s+da\s+descarga\s+s.lida|Einstein\s+Modificado|Colby\s+Simplificado</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="F49" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Tema descarga liquida/vazao.</t>
+          <t>Regra desativada: DSL pode mencionar planilhas de descarga solida no corpo do relatorio.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>template_laudo_dsl_v1</t>
+          <t>template_laudo_dss_v1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>required</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -6290,25 +6092,25 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>ADCP|Tipo\s+de\s+medidor|Dados\s+do\s+equipamento</t>
+          <t>RELAT.RIO\s+DE\s+ENSAIO|Relat.rio\s+de\s+Ensaio</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Equipamento e metodologia de DSL.</t>
+          <t>Documento deve ser relatorio de ensaio.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>template_laudo_dsl_v1</t>
+          <t>template_laudo_dss_v1</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -6323,25 +6125,25 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Determina..o\s+da\s+descarga\s+l.quida</t>
+          <t>Medi..o\s+de\s+Descarga\s+S.lida|Descarga\s+S.lida</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F51" t="b">
         <v>1</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Metodologia declarada de DSL.</t>
+          <t>Tema descarga solida.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>template_laudo_dsl_v1</t>
+          <t>template_laudo_dss_v1</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6351,35 +6153,35 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>path</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>(?:\|/|_)DSL(?:\|/|_|\.)</t>
+          <t>Einstein\s+Modificado|Colby\s+Simplificado</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F52" t="b">
         <v>1</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Caminho ou nome indica DSL.</t>
+          <t>Metodologias caracteristicas de DSS.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>template_laudo_dsl_v1</t>
+          <t>template_laudo_dss_v1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -6389,18 +6191,18 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Medi..o\s+de\s+Descarga\s+S.lida|Determina..o\s+da\s+descarga\s+s.lida|Einstein\s+Modificado|Colby\s+Simplificado</t>
+          <t>Dados\s+de\s+Entrada|DADOS\s+D</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Regra desativada: DSL pode mencionar planilhas de descarga solida no corpo do relatorio.</t>
+          <t>Secao de entrada caracteristica de DSS.</t>
         </is>
       </c>
     </row>
@@ -6412,7 +6214,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>required</t>
+          <t>negative</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -6422,7 +6224,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>RELAT.RIO\s+DE\s+ENSAIO|Relat.rio\s+de\s+Ensaio</t>
+          <t>Descarga\s+L.quida|ADCP</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -6433,19 +6235,19 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Documento deve ser relatorio de ensaio.</t>
+          <t>Regra desativada: DSS tambem pode citar descarga liquida/ADCP como dado de entrada.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>template_laudo_dss_v1</t>
+          <t>template_ficha_coleta_tommasi_v1</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>required</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -6455,25 +6257,25 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Medi..o\s+de\s+Descarga\s+S.lida|Descarga\s+S.lida</t>
+          <t>Cadeia\s+de\s+Cust.dia</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F55" t="b">
         <v>1</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Tema descarga solida.</t>
+          <t>Documento deve ser cadeia de custodia.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>template_laudo_dss_v1</t>
+          <t>template_ficha_coleta_tommasi_v1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -6488,25 +6290,25 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Einstein\s+Modificado|Colby\s+Simplificado</t>
+          <t>Amostra\s+Id|Identifica..o\s+ou\s+Ponto\s+de\s+Coleta</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="F56" t="b">
         <v>1</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Metodologias caracteristicas de DSS.</t>
+          <t>Campos caracteristicos da ficha de coleta Tommasi.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>template_laudo_dss_v1</t>
+          <t>template_ficha_coleta_tommasi_v1</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -6521,25 +6323,25 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Dados\s+de\s+Entrada|DADOS\s+D</t>
+          <t>Embalagem\s+e\s+Preserva..o|Planejamento\s+de\s+Amostragem</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F57" t="b">
         <v>1</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Secao de entrada caracteristica de DSS.</t>
+          <t>Campos de embalagem/planejamento de coleta.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>template_laudo_dss_v1</t>
+          <t>template_ficha_coleta_tommasi_v1</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -6549,12 +6351,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>path</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>(?:\|/|_)DSS(?:\|/|_|\.)</t>
+          <t>Checklist\s+de\s+recebimento|Data\s+e\s+Hora\s+de\s+Recebimento</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -6565,14 +6367,14 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Caminho ou nome indica DSS.</t>
+          <t>Checklist de recebimento acoplado a COC.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>template_laudo_dss_v1</t>
+          <t>template_ficha_coleta_tommasi_v1</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -6587,25 +6389,25 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Descarga\s+L.quida|ADCP</t>
+          <t>Relat.rio\s+Anal.tico|Relat.rio\s+de\s+Ensaio|Confirma..o\s+de\s+Recebimento</t>
         </is>
       </c>
       <c r="E59" t="n">
         <v>0</v>
       </c>
       <c r="F59" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Regra desativada: DSS tambem pode citar descarga liquida/ADCP como dado de entrada.</t>
+          <t>Evita confundir ficha com laudos ou recebimentos subcontratados.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>template_ficha_coleta_tommasi_v1</t>
+          <t>template_ficha_recebimento_aplysia_v1</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -6620,7 +6422,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Cadeia\s+de\s+Cust.dia</t>
+          <t>Confirma..o\s+de\s+Recebimento\s+de\s+Amostras</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -6631,14 +6433,14 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Documento deve ser cadeia de custodia.</t>
+          <t>Documento de confirmacao de recebimento.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>template_ficha_coleta_tommasi_v1</t>
+          <t>template_ficha_recebimento_aplysia_v1</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -6653,7 +6455,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Amostra\s+Id|Identifica..o\s+ou\s+Ponto\s+de\s+Coleta</t>
+          <t>APLYSIA</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -6664,14 +6466,14 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Campos caracteristicos da ficha de coleta Tommasi.</t>
+          <t>Laboratorio Aplysia.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>template_ficha_coleta_tommasi_v1</t>
+          <t>template_ficha_recebimento_aplysia_v1</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -6686,30 +6488,30 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Embalagem\s+e\s+Preserva..o|Planejamento\s+de\s+Amostragem</t>
+          <t>Ensaios?\s+Ecotoxicol.gicos?|Daphnia|Ceriodaphnia|Hyalella|Raphidocelis</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="F62" t="b">
         <v>1</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Campos de embalagem/planejamento de coleta.</t>
+          <t>Ensaios/organismos de ecotoxicologia.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>template_ficha_coleta_tommasi_v1</t>
+          <t>template_ficha_recebimento_labmar_v1</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>required</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -6719,25 +6521,25 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Checklist\s+de\s+recebimento|Data\s+e\s+Hora\s+de\s+Recebimento</t>
+          <t>Checklist\s+de\s+Recebimento</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F63" t="b">
         <v>1</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Checklist de recebimento acoplado a COC.</t>
+          <t>Documento checklist de recebimento.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>template_ficha_coleta_tommasi_v1</t>
+          <t>template_ficha_recebimento_labmar_v1</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -6747,35 +6549,35 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>path</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Fichas\s+de\s+coleta</t>
+          <t>LABMAR|FM-LAB-035|LAUDO\s+VINCULADO</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="F64" t="b">
         <v>1</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Caminho indica ficha de coleta.</t>
+          <t>Formato Labmar.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>template_ficha_coleta_tommasi_v1</t>
+          <t>template_ficha_recebimento_labmar_v1</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -6785,25 +6587,25 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Relat.rio\s+Anal.tico|Relat.rio\s+de\s+Ensaio|Confirma..o\s+de\s+Recebimento</t>
+          <t>N.?\s*PROPOSTA\s+COMERCIAL|DATA\s+DO\s+RECEBIMENTO</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F65" t="b">
         <v>1</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Evita confundir ficha com laudos ou recebimentos subcontratados.</t>
+          <t>Campos caracteristicos de recebimento Labmar.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_aplysia_v1</t>
+          <t>template_ficha_recebimento_ethica_v1</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -6818,25 +6620,25 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Confirma..o\s+de\s+Recebimento\s+de\s+Amostras</t>
+          <t>RESPONS.VEL\s+PELA\s+ENTREGA|RESPONS.VEL\s+PELO\s+RECEBIMENTO</t>
         </is>
       </c>
       <c r="E66" t="n">
         <v>0</v>
       </c>
       <c r="F66" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Documento de confirmacao de recebimento.</t>
+          <t>Regra desativada: alguns checklists Ethica nao possuem texto extraivel; caminho forte assume a identificacao.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_aplysia_v1</t>
+          <t>template_ficha_recebimento_ethica_v1</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -6851,25 +6653,25 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>APLYSIA</t>
+          <t>ID\s+Amostra\s+Data\s*/\s*Hora\s+Coleta|Proposta\s+.*Comercial</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F67" t="b">
         <v>1</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Laboratorio Aplysia.</t>
+          <t>Cabecalho tabular Ethica.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_aplysia_v1</t>
+          <t>template_ficha_recebimento_ethica_v1</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -6884,25 +6686,25 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Ensaios?\s+Ecotoxicol.gicos?|Daphnia|Ceriodaphnia|Hyalella|Raphidocelis</t>
+          <t>Clorofila\s+e\s+Feofitina|Preservante|Refrigerado</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F68" t="b">
         <v>1</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Ensaios/organismos de ecotoxicologia.</t>
+          <t>Campos/analises caracteristicas do recebimento Ethica.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_aplysia_v1</t>
+          <t>template_laudo_zbt_v1</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -6912,35 +6714,35 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>path</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Aplysia</t>
+          <t>Meiofauna\s+Bent.nica|Meiofauna\s+de\s+fundo</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="F69" t="b">
         <v>1</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Caminho indica Aplysia.</t>
+          <t>Reconhece laudos ZBT de meiofauna bentonica.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_labmar_v1</t>
+          <t>template_laudo_sedimento_v1</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>required</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -6950,30 +6752,30 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Checklist\s+de\s+Recebimento</t>
+          <t>Sedimento\s*-\s*Branco\s+de\s+equipamento|Sedimento\s*-\s*Branco</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F70" t="b">
         <v>1</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Documento checklist de recebimento.</t>
+          <t>Reconhece branco de equipamento associado a sedimento.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_labmar_v1</t>
+          <t>template_ficha_subcontratacao_als_v1</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>required</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -6983,25 +6785,25 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>LABMAR|FM-LAB-035|LAUDO\s+VINCULADO</t>
+          <t>SUBCONTRATA..O\s+DE\s+SERVI.OS\s+DE\s+AN.LISE|FO-ANL-098</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F71" t="b">
         <v>1</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Formato Labmar.</t>
+          <t>Documento de subcontratacao de servicos de analise.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_labmar_v1</t>
+          <t>template_ficha_subcontratacao_als_v1</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -7016,25 +6818,25 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>N.?\s*PROPOSTA\s+COMERCIAL|DATA\s+DO\s+RECEBIMENTO</t>
+          <t>Provedor\s+Externo:\s*ALS|ALS\s+Corplab</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="F72" t="b">
         <v>1</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Campos caracteristicos de recebimento Labmar.</t>
+          <t>Provedor externo ALS Corplab.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_labmar_v1</t>
+          <t>template_ficha_subcontratacao_als_v1</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -7044,35 +6846,35 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>path</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Labmar</t>
+          <t>ID\s+Amostra\s+Identifica..o\s+Data/Hora\s+Coleta|Matriz\s+An.lise\s+Metodologia</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F73" t="b">
         <v>1</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Caminho indica Labmar.</t>
+          <t>Cabecalho tabular da ficha ALS.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_ethica_v1</t>
+          <t>template_ficha_subcontratacao_als_v1</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>required</t>
+          <t>negative</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -7082,30 +6884,30 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>RESPONS.VEL\s+PELA\s+ENTREGA|RESPONS.VEL\s+PELO\s+RECEBIMENTO</t>
+          <t>Relat.rio\s+Anal.tico|Relat.rio\s+de\s+Ensaio|Cadeia\s+de\s+Cust.dia</t>
         </is>
       </c>
       <c r="E74" t="n">
         <v>0</v>
       </c>
       <c r="F74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Regra desativada: alguns checklists Ethica nao possuem texto extraivel; caminho forte assume a identificacao.</t>
+          <t>Evita confundir ficha ALS com laudos ou COC principal.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_ethica_v1</t>
+          <t>template_ficha_recebimento_bioagri_v1</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>negative</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -7115,25 +6917,25 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>ID\s+Amostra\s+Data\s*/\s*Hora\s+Coleta|Proposta\s+.*Comercial</t>
+          <t>Relat.rio\s+Anal.tico|Relat.rio\s+de\s+Ensaio|Cadeia\s+de\s+Cust.dia</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="F75" t="b">
         <v>1</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Cabecalho tabular Ethica.</t>
+          <t>Evita confundir checklist Bioagri com laudos ou COC principal.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_ethica_v1</t>
+          <t>template_ficha_recebimento_bioagri_v1</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -7148,25 +6950,25 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Clorofila\s+e\s+Feofitina|Preservante|Refrigerado</t>
+          <t>Bioagri|Eurofins</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F76" t="b">
         <v>1</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Campos/analises caracteristicas do recebimento Ethica.</t>
+          <t>Identifica fornecedor/laboratorio Bioagri no texto.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_ethica_v1</t>
+          <t>template_ficha_recebimento_bioagri_v1</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -7176,30 +6978,30 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>path</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>.thica|Ethica</t>
+          <t>Checklist\s+de\s+Recebimento|Recebimento\s+de\s+Amostras</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F77" t="b">
         <v>1</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Caminho indica Ethica.</t>
+          <t>Estrutura textual de checklist/recebimento Bioagri.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>template_laudo_zbt_v1</t>
+          <t>template_ficha_recebimento_bioagri_v1</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -7214,447 +7016,18 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Meiofauna\s+Bent.nica|Meiofauna\s+de\s+fundo</t>
+          <t>Condi..es\s+de\s+recebimento|Amostras?\s+recebidas?|Temperatura\s+de\s+recebimento</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="F78" t="b">
         <v>1</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Reconhece laudos ZBT de meiofauna bentonica.</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>template_laudo_sedimento_v1</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>path</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>(?:\|/|_)Sed(?:\|/|_|\.)</t>
-        </is>
-      </c>
-      <c r="E79" t="n">
-        <v>40</v>
-      </c>
-      <c r="F79" t="b">
-        <v>1</v>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>Caminho ou nome indica laudo de sedimento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>template_laudo_sedimento_v1</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Sedimento\s*-\s*Branco\s+de\s+equipamento|Sedimento\s*-\s*Branco</t>
-        </is>
-      </c>
-      <c r="E80" t="n">
-        <v>40</v>
-      </c>
-      <c r="F80" t="b">
-        <v>1</v>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>Reconhece branco de equipamento associado a sedimento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>template_ficha_subcontratacao_als_v1</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>required</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>SUBCONTRATA..O\s+DE\s+SERVI.OS\s+DE\s+AN.LISE|FO-ANL-098</t>
-        </is>
-      </c>
-      <c r="E81" t="n">
-        <v>0</v>
-      </c>
-      <c r="F81" t="b">
-        <v>1</v>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>Documento de subcontratacao de servicos de analise.</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>template_ficha_subcontratacao_als_v1</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Provedor\s+Externo:\s*ALS|ALS\s+Corplab</t>
-        </is>
-      </c>
-      <c r="E82" t="n">
-        <v>50</v>
-      </c>
-      <c r="F82" t="b">
-        <v>1</v>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>Provedor externo ALS Corplab.</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>template_ficha_subcontratacao_als_v1</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>ID\s+Amostra\s+Identifica..o\s+Data/Hora\s+Coleta|Matriz\s+An.lise\s+Metodologia</t>
-        </is>
-      </c>
-      <c r="E83" t="n">
-        <v>30</v>
-      </c>
-      <c r="F83" t="b">
-        <v>1</v>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>Cabecalho tabular da ficha ALS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>template_ficha_subcontratacao_als_v1</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>path</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>COC_subcontratadas.*ALS|ALS</t>
-        </is>
-      </c>
-      <c r="E84" t="n">
-        <v>30</v>
-      </c>
-      <c r="F84" t="b">
-        <v>1</v>
-      </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>Caminho indica subcontratada ALS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>template_ficha_subcontratacao_als_v1</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>negative</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Relat.rio\s+Anal.tico|Relat.rio\s+de\s+Ensaio|Cadeia\s+de\s+Cust.dia</t>
-        </is>
-      </c>
-      <c r="E85" t="n">
-        <v>0</v>
-      </c>
-      <c r="F85" t="b">
-        <v>1</v>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>Evita confundir ficha ALS com laudos ou COC principal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>template_ficha_recebimento_bioagri_v1</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>path</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>COC_subcontratadas.*Bioagri|Bioagri</t>
-        </is>
-      </c>
-      <c r="E86" t="n">
-        <v>85</v>
-      </c>
-      <c r="F86" t="b">
-        <v>1</v>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>Caminho indica recebimento/checklist Bioagri.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>template_ficha_recebimento_bioagri_v1</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>path</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>Checklist\s+de\s+Recebimento</t>
-        </is>
-      </c>
-      <c r="E87" t="n">
-        <v>20</v>
-      </c>
-      <c r="F87" t="b">
-        <v>1</v>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>Nome do arquivo indica checklist de recebimento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>template_ficha_recebimento_bioagri_v1</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>negative</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>Relat.rio\s+Anal.tico|Relat.rio\s+de\s+Ensaio|Cadeia\s+de\s+Cust.dia</t>
-        </is>
-      </c>
-      <c r="E88" t="n">
-        <v>0</v>
-      </c>
-      <c r="F88" t="b">
-        <v>1</v>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>Evita confundir checklist Bioagri com laudos ou COC principal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>template_ficha_recebimento_ethica_v1</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>path</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>COC_subcontratadas.*(?:.thica|Ethica)</t>
-        </is>
-      </c>
-      <c r="E89" t="n">
-        <v>85</v>
-      </c>
-      <c r="F89" t="b">
-        <v>1</v>
-      </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>Caminho forte indica recebimento Ethica em subcontratadas, inclusive em PDF sem texto extraivel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>template_laudo_zbt_v1</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>path</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>\\ZBT\\|/ZBT/|_bentos\.pdf|bentos</t>
-        </is>
-      </c>
-      <c r="E90" t="n">
-        <v>90</v>
-      </c>
-      <c r="F90" t="b">
-        <v>1</v>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>Caminho ou nome indica laudo ZBT/bentos quando o PDF nao tem texto extraivel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>template_laudo_dss_v1</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>path</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>\\DSS\\|/DSS/</t>
-        </is>
-      </c>
-      <c r="E91" t="n">
-        <v>90</v>
-      </c>
-      <c r="F91" t="b">
-        <v>1</v>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>Caminho indica laudo DSS quando o PDF nao tem texto extraivel.</t>
+          <t>Campos textuais caracteristicos de recebimento Bioagri.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Normalize result layouts taxonomy
</commit_message>
<xml_diff>
--- a/config/taxonomy_config_v5.xlsx
+++ b/config/taxonomy_config_v5.xlsx
@@ -11337,7 +11337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11353,70 +11353,15 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>resultado_col</t>
+          <t>campo</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>unidade_col</t>
+          <t>coluna_origem</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
-        <is>
-          <t>data_inicio_col</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>criterio_conformidade_col</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>lq_col</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>referencia_col</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>incerteza_col</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>numero_cq_col</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>duplicata_col</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>faixa_aceitacao_col</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>variacao_percentual_col</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>quantidade_adicionada_col</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>recuperacao_percentual_col</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
@@ -11433,25 +11378,15 @@
           <t>AMOSTRA</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I2" t="n">
-        <v>6</v>
-      </c>
-      <c r="P2" t="b">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -11463,22 +11398,18 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BRANCO</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
+          <t>AMOSTRA</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>data_inicio</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>2</v>
       </c>
-      <c r="D3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
-      <c r="P3" t="b">
+      <c r="E3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -11490,28 +11421,18 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DUPLICATA</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>2</v>
+          <t>AMOSTRA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>criterio_conformidade</t>
+        </is>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" t="n">
         <v>3</v>
       </c>
-      <c r="L4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M4" t="n">
-        <v>6</v>
-      </c>
-      <c r="P4" t="b">
+      <c r="E4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -11523,28 +11444,432 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>AMOSTRA</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>lq</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AMOSTRA</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>referencia</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AMOSTRA</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>incerteza</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BRANCO</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BRANCO</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>unidade</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BRANCO</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>lq</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BRANCO</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>numero_cq</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DUPLICATA</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>DUPLICATA</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>unidade</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>DUPLICATA</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>numero_cq</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>DUPLICATA</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>duplicata</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>DUPLICATA</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>faixa_aceitacao</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>DUPLICATA</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>variacao_percentual</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>RECUPERACAO</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
         <v>5</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>RECUPERACAO</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>unidade</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
         <v>3</v>
       </c>
-      <c r="J5" t="n">
-        <v>1</v>
-      </c>
-      <c r="L5" t="n">
+      <c r="E19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>RECUPERACAO</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>numero_cq</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>RECUPERACAO</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>faixa_aceitacao</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
         <v>4</v>
       </c>
-      <c r="N5" t="n">
+      <c r="E21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>RECUPERACAO</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>quantidade_adicionada</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
         <v>2</v>
       </c>
-      <c r="O5" t="n">
+      <c r="E22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>RECUPERACAO</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>recuperacao_percentual</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
         <v>5</v>
       </c>
-      <c r="P5" t="b">
+      <c r="E23" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Standardize taxonomy boolean fields
</commit_message>
<xml_diff>
--- a/config/taxonomy_config_v5.xlsx
+++ b/config/taxonomy_config_v5.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="10" activeTab="12" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="templates" sheetId="1" state="visible" r:id="rId1"/>
@@ -22,7 +21,7 @@
     <sheet name="client_output_schema" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -62,7 +61,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -426,7 +425,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -986,7 +985,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1082,7 +1081,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="11.7265625" bestFit="1" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1140,10 +1142,8 @@
           <t>texto</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
+      <c r="E2" t="b">
+        <v>1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1175,10 +1175,8 @@
           <t>texto</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
+      <c r="E3" t="b">
+        <v>1</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1210,10 +1208,8 @@
           <t>texto</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>nao</t>
-        </is>
+      <c r="E4" t="b">
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -2228,7 +2224,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="11.7265625" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="26.54296875" bestFit="1" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2286,10 +2286,8 @@
           <t>texto</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
+      <c r="E2" t="b">
+        <v>1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2321,10 +2319,8 @@
           <t>texto</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
+      <c r="E3" t="b">
+        <v>1</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2356,10 +2352,8 @@
           <t>texto</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>nao</t>
-        </is>
+      <c r="E4" t="b">
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -3077,7 +3071,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3135,10 +3129,8 @@
           <t>texto</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
+      <c r="E2" t="b">
+        <v>1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3170,10 +3162,8 @@
           <t>texto</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
+      <c r="E3" t="b">
+        <v>1</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3205,10 +3195,8 @@
           <t>texto</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>nao</t>
-        </is>
+      <c r="E4" t="b">
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -3464,7 +3452,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G78"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="11.7265625" bestFit="1" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -6056,7 +6047,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F71"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -8062,7 +8053,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="11.7265625" bestFit="1" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -8398,7 +8392,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -8964,7 +8958,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D49"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -9960,7 +9954,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F38"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -11042,7 +11036,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="11.7265625" bestFit="1" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -11338,7 +11335,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="22.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="13.26953125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="21.36328125" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="13.26953125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="11.7265625" bestFit="1" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>

<commit_message>
Add generic table extraction audit
</commit_message>
<xml_diff>
--- a/config/taxonomy_config_v5.xlsx
+++ b/config/taxonomy_config_v5.xlsx
@@ -25,7 +25,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'templates'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'template_detection_rules'!$A$1:$G$78</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'output_sheets'!$A$1:$F$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'output_sheets'!$A$1:$F$85</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'metadata_schema'!$A$1:$D$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'client_schema'!$A$1:$E$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'sample_schema'!$A$1:$D$49</definedName>
@@ -6850,15 +6850,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="49" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6896,12 +6896,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>template_laudo_agua_v1</t>
+          <t>template_ficha_coleta_tommasi_v1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>laudo_agua</t>
+          <t>ficha_coleta_tommasi</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -6924,12 +6924,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>template_laudo_agua_v1</t>
+          <t>template_ficha_coleta_tommasi_v1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>laudo_agua</t>
+          <t>ficha_coleta_tommasi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -6952,12 +6952,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>template_laudo_agua_v1</t>
+          <t>template_ficha_coleta_tommasi_v1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>laudo_agua</t>
+          <t>ficha_coleta_tommasi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -6980,712 +6980,712 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>template_laudo_agua_v1</t>
+          <t>template_ficha_coleta_tommasi_v1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>laudo_agua</t>
+          <t>ficha_coleta_tommasi</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>table_extraction_audit</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>template_laudo_agua_v1</t>
+          <t>template_ficha_coleta_tommasi_v1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>laudo_agua</t>
+          <t>ficha_coleta_tommasi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>validation_errors</t>
+          <t>classification_audit</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Erros de validacao da saida.</t>
+          <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>template_laudo_fito_v1</t>
+          <t>template_ficha_coleta_tommasi_v1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>laudo_fito</t>
+          <t>ficha_coleta_tommasi</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>results_extract</t>
+          <t>validation_errors</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Resultados extraidos do PDF para o template.</t>
+          <t>Erros de validacao da saida.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>template_laudo_fito_v1</t>
+          <t>template_ficha_recebimento_aplysia_v1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>laudo_fito</t>
+          <t>ficha_recebimento_aplysia</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>template_laudo_fito_v1</t>
+          <t>template_ficha_recebimento_aplysia_v1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>laudo_fito</t>
+          <t>ficha_recebimento_aplysia</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>template_laudo_fito_v1</t>
+          <t>template_ficha_recebimento_aplysia_v1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>laudo_fito</t>
+          <t>ficha_recebimento_aplysia</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>client</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>98</v>
+        <v>3</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Dados de identificacao do cliente.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>template_laudo_fito_v1</t>
+          <t>template_ficha_recebimento_aplysia_v1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>laudo_fito</t>
+          <t>ficha_recebimento_aplysia</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>validation_errors</t>
+          <t>table_extraction_audit</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E11" t="b">
         <v>1</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Erros de validacao da saida.</t>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>template_laudo_sedimento_v1</t>
+          <t>template_ficha_recebimento_aplysia_v1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>laudo_sedimento</t>
+          <t>ficha_recebimento_aplysia</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>results_extract</t>
+          <t>classification_audit</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>98</v>
       </c>
       <c r="E12" t="b">
         <v>1</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Resultados extraidos do PDF para o template.</t>
+          <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>template_laudo_sedimento_v1</t>
+          <t>template_ficha_recebimento_aplysia_v1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>laudo_sedimento</t>
+          <t>ficha_recebimento_aplysia</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>validation_errors</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>99</v>
       </c>
       <c r="E13" t="b">
         <v>1</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Erros de validacao da saida.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>template_laudo_sedimento_v1</t>
+          <t>template_ficha_recebimento_bioagri_v1</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>laudo_sedimento</t>
+          <t>ficha_recebimento_bioagri</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E14" t="b">
         <v>1</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>template_laudo_sedimento_v1</t>
+          <t>template_ficha_recebimento_bioagri_v1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>laudo_sedimento</t>
+          <t>ficha_recebimento_bioagri</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>98</v>
+        <v>2</v>
       </c>
       <c r="E15" t="b">
         <v>1</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>template_laudo_sedimento_v1</t>
+          <t>template_ficha_recebimento_bioagri_v1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>laudo_sedimento</t>
+          <t>ficha_recebimento_bioagri</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>validation_errors</t>
+          <t>client</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>99</v>
+        <v>3</v>
       </c>
       <c r="E16" t="b">
         <v>1</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Erros de validacao da saida.</t>
+          <t>Dados de identificacao do cliente.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>template_laudo_mps_v1</t>
+          <t>template_ficha_recebimento_bioagri_v1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>laudo_mps</t>
+          <t>ficha_recebimento_bioagri</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>results_extract</t>
+          <t>table_extraction_audit</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>97</v>
       </c>
       <c r="E17" t="b">
         <v>1</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Resultados extraidos do PDF para o template.</t>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>template_laudo_mps_v1</t>
+          <t>template_ficha_recebimento_bioagri_v1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>laudo_mps</t>
+          <t>ficha_recebimento_bioagri</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>classification_audit</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>98</v>
       </c>
       <c r="E18" t="b">
         <v>1</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>template_laudo_mps_v1</t>
+          <t>template_ficha_recebimento_bioagri_v1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>laudo_mps</t>
+          <t>ficha_recebimento_bioagri</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>validation_errors</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>99</v>
       </c>
       <c r="E19" t="b">
         <v>1</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Erros de validacao da saida.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>template_laudo_mps_v1</t>
+          <t>template_ficha_recebimento_ethica_v1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>laudo_mps</t>
+          <t>ficha_recebimento_ethica</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>98</v>
+        <v>1</v>
       </c>
       <c r="E20" t="b">
         <v>1</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>template_laudo_mps_v1</t>
+          <t>template_ficha_recebimento_ethica_v1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>laudo_mps</t>
+          <t>ficha_recebimento_ethica</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>validation_errors</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>99</v>
+        <v>2</v>
       </c>
       <c r="E21" t="b">
         <v>1</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Erros de validacao da saida.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>template_laudo_ect_v1</t>
+          <t>template_ficha_recebimento_ethica_v1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>laudo_ect</t>
+          <t>ficha_recebimento_ethica</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>results_extract</t>
+          <t>client</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E22" t="b">
         <v>1</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Resultados extraidos do PDF para o template.</t>
+          <t>Dados de identificacao do cliente.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>template_laudo_ect_v1</t>
+          <t>template_ficha_recebimento_ethica_v1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>laudo_ect</t>
+          <t>ficha_recebimento_ethica</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>table_extraction_audit</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>2</v>
+        <v>97</v>
       </c>
       <c r="E23" t="b">
         <v>1</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>template_laudo_ect_v1</t>
+          <t>template_ficha_recebimento_ethica_v1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>laudo_ect</t>
+          <t>ficha_recebimento_ethica</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>classification_audit</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3</v>
+        <v>98</v>
       </c>
       <c r="E24" t="b">
         <v>1</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>template_laudo_ect_v1</t>
+          <t>template_ficha_recebimento_ethica_v1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>laudo_ect</t>
+          <t>ficha_recebimento_ethica</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>validation_errors</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E25" t="b">
         <v>1</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Erros de validacao da saida.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>template_laudo_ect_v1</t>
+          <t>template_ficha_recebimento_labmar_v1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>laudo_ect</t>
+          <t>ficha_recebimento_labmar</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>validation_errors</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="E26" t="b">
         <v>1</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Erros de validacao da saida.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>template_laudo_zbt_v1</t>
+          <t>template_ficha_recebimento_labmar_v1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>laudo_zbt</t>
+          <t>ficha_recebimento_labmar</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>results_extract</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E27" t="b">
         <v>1</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Resultados extraidos do PDF para o template.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>template_laudo_zbt_v1</t>
+          <t>template_ficha_recebimento_labmar_v1</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>laudo_zbt</t>
+          <t>ficha_recebimento_labmar</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>client</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E28" t="b">
         <v>1</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Dados de identificacao do cliente.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>template_laudo_zbt_v1</t>
+          <t>template_ficha_recebimento_labmar_v1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>laudo_zbt</t>
+          <t>ficha_recebimento_labmar</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>table_extraction_audit</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="E29" t="b">
         <v>1</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>template_laudo_zbt_v1</t>
+          <t>template_ficha_recebimento_labmar_v1</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>laudo_zbt</t>
+          <t>ficha_recebimento_labmar</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -7708,12 +7708,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>template_laudo_zbt_v1</t>
+          <t>template_ficha_recebimento_labmar_v1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>laudo_zbt</t>
+          <t>ficha_recebimento_labmar</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -7736,12 +7736,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>template_laudo_dsl_v1</t>
+          <t>template_ficha_subcontratacao_als_v1</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>laudo_dsl</t>
+          <t>ficha_subcontratacao_als</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -7764,12 +7764,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>template_laudo_dsl_v1</t>
+          <t>template_ficha_subcontratacao_als_v1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>laudo_dsl</t>
+          <t>ficha_subcontratacao_als</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -7792,12 +7792,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>template_laudo_dsl_v1</t>
+          <t>template_ficha_subcontratacao_als_v1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>laudo_dsl</t>
+          <t>ficha_subcontratacao_als</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -7820,712 +7820,712 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>template_laudo_dsl_v1</t>
+          <t>template_ficha_subcontratacao_als_v1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>laudo_dsl</t>
+          <t>ficha_subcontratacao_als</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>table_extraction_audit</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E35" t="b">
         <v>1</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>template_laudo_dsl_v1</t>
+          <t>template_ficha_subcontratacao_als_v1</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>laudo_dsl</t>
+          <t>ficha_subcontratacao_als</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>validation_errors</t>
+          <t>classification_audit</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E36" t="b">
         <v>1</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Erros de validacao da saida.</t>
+          <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>template_laudo_dss_v1</t>
+          <t>template_ficha_subcontratacao_als_v1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>laudo_dss</t>
+          <t>ficha_subcontratacao_als</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>results_extract</t>
+          <t>validation_errors</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="E37" t="b">
         <v>1</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Resultados extraidos do PDF para o template.</t>
+          <t>Erros de validacao da saida.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>template_laudo_dss_v1</t>
+          <t>template_laudo_agua_v1</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>laudo_dss</t>
+          <t>laudo_agua</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E38" t="b">
         <v>1</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>template_laudo_dss_v1</t>
+          <t>template_laudo_agua_v1</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>laudo_dss</t>
+          <t>laudo_agua</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E39" t="b">
         <v>1</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>template_laudo_dss_v1</t>
+          <t>template_laudo_agua_v1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>laudo_dss</t>
+          <t>laudo_agua</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>client</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>98</v>
+        <v>3</v>
       </c>
       <c r="E40" t="b">
         <v>1</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Dados de identificacao do cliente.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>template_laudo_dss_v1</t>
+          <t>template_laudo_agua_v1</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>laudo_dss</t>
+          <t>laudo_agua</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>validation_errors</t>
+          <t>table_extraction_audit</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E41" t="b">
         <v>1</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Erros de validacao da saida.</t>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>template_ficha_coleta_tommasi_v1</t>
+          <t>template_laudo_agua_v1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ficha_coleta_tommasi</t>
+          <t>laudo_agua</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>results_extract</t>
+          <t>classification_audit</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>1</v>
+        <v>98</v>
       </c>
       <c r="E42" t="b">
         <v>1</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Resultados extraidos do PDF para o template.</t>
+          <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>template_ficha_coleta_tommasi_v1</t>
+          <t>template_laudo_agua_v1</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ficha_coleta_tommasi</t>
+          <t>laudo_agua</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>validation_errors</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2</v>
+        <v>99</v>
       </c>
       <c r="E43" t="b">
         <v>1</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Erros de validacao da saida.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>template_ficha_coleta_tommasi_v1</t>
+          <t>template_laudo_dsl_v1</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ficha_coleta_tommasi</t>
+          <t>laudo_dsl</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E44" t="b">
         <v>1</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>template_ficha_coleta_tommasi_v1</t>
+          <t>template_laudo_dsl_v1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ficha_coleta_tommasi</t>
+          <t>laudo_dsl</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>98</v>
+        <v>2</v>
       </c>
       <c r="E45" t="b">
         <v>1</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>template_ficha_coleta_tommasi_v1</t>
+          <t>template_laudo_dsl_v1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ficha_coleta_tommasi</t>
+          <t>laudo_dsl</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>validation_errors</t>
+          <t>client</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>99</v>
+        <v>3</v>
       </c>
       <c r="E46" t="b">
         <v>1</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Erros de validacao da saida.</t>
+          <t>Dados de identificacao do cliente.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_aplysia_v1</t>
+          <t>template_laudo_dsl_v1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ficha_recebimento_aplysia</t>
+          <t>laudo_dsl</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>results_extract</t>
+          <t>table_extraction_audit</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1</v>
+        <v>97</v>
       </c>
       <c r="E47" t="b">
         <v>1</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Resultados extraidos do PDF para o template.</t>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_aplysia_v1</t>
+          <t>template_laudo_dsl_v1</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ficha_recebimento_aplysia</t>
+          <t>laudo_dsl</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>classification_audit</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>2</v>
+        <v>98</v>
       </c>
       <c r="E48" t="b">
         <v>1</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_aplysia_v1</t>
+          <t>template_laudo_dsl_v1</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ficha_recebimento_aplysia</t>
+          <t>laudo_dsl</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>validation_errors</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>3</v>
+        <v>99</v>
       </c>
       <c r="E49" t="b">
         <v>1</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Erros de validacao da saida.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_aplysia_v1</t>
+          <t>template_laudo_dss_v1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ficha_recebimento_aplysia</t>
+          <t>laudo_dss</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>98</v>
+        <v>1</v>
       </c>
       <c r="E50" t="b">
         <v>1</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_aplysia_v1</t>
+          <t>template_laudo_dss_v1</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ficha_recebimento_aplysia</t>
+          <t>laudo_dss</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>validation_errors</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>99</v>
+        <v>2</v>
       </c>
       <c r="E51" t="b">
         <v>1</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Erros de validacao da saida.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_labmar_v1</t>
+          <t>template_laudo_dss_v1</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ficha_recebimento_labmar</t>
+          <t>laudo_dss</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>results_extract</t>
+          <t>client</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E52" t="b">
         <v>1</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Resultados extraidos do PDF para o template.</t>
+          <t>Dados de identificacao do cliente.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_labmar_v1</t>
+          <t>template_laudo_dss_v1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ficha_recebimento_labmar</t>
+          <t>laudo_dss</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>table_extraction_audit</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>2</v>
+        <v>97</v>
       </c>
       <c r="E53" t="b">
         <v>1</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_labmar_v1</t>
+          <t>template_laudo_dss_v1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ficha_recebimento_labmar</t>
+          <t>laudo_dss</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>classification_audit</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>3</v>
+        <v>98</v>
       </c>
       <c r="E54" t="b">
         <v>1</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_labmar_v1</t>
+          <t>template_laudo_dss_v1</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ficha_recebimento_labmar</t>
+          <t>laudo_dss</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>validation_errors</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E55" t="b">
         <v>1</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Erros de validacao da saida.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_labmar_v1</t>
+          <t>template_laudo_ect_v1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ficha_recebimento_labmar</t>
+          <t>laudo_ect</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>validation_errors</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="E56" t="b">
         <v>1</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Erros de validacao da saida.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_ethica_v1</t>
+          <t>template_laudo_ect_v1</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ficha_recebimento_ethica</t>
+          <t>laudo_ect</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>results_extract</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E57" t="b">
         <v>1</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Resultados extraidos do PDF para o template.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_ethica_v1</t>
+          <t>template_laudo_ect_v1</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ficha_recebimento_ethica</t>
+          <t>laudo_ect</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>client</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E58" t="b">
         <v>1</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Dados de identificacao do cliente.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_ethica_v1</t>
+          <t>template_laudo_ect_v1</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ficha_recebimento_ethica</t>
+          <t>laudo_ect</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>table_extraction_audit</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="E59" t="b">
         <v>1</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_ethica_v1</t>
+          <t>template_laudo_ect_v1</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ficha_recebimento_ethica</t>
+          <t>laudo_ect</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -8548,12 +8548,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_ethica_v1</t>
+          <t>template_laudo_ect_v1</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ficha_recebimento_ethica</t>
+          <t>laudo_ect</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -8576,12 +8576,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>template_ficha_subcontratacao_als_v1</t>
+          <t>template_laudo_fito_v1</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ficha_subcontratacao_als</t>
+          <t>laudo_fito</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -8604,12 +8604,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>template_ficha_subcontratacao_als_v1</t>
+          <t>template_laudo_fito_v1</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ficha_subcontratacao_als</t>
+          <t>laudo_fito</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -8632,12 +8632,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>template_ficha_subcontratacao_als_v1</t>
+          <t>template_laudo_fito_v1</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ficha_subcontratacao_als</t>
+          <t>laudo_fito</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -8660,201 +8660,593 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>template_ficha_subcontratacao_als_v1</t>
+          <t>template_laudo_fito_v1</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ficha_subcontratacao_als</t>
+          <t>laudo_fito</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>table_extraction_audit</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E65" t="b">
         <v>1</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>template_ficha_subcontratacao_als_v1</t>
+          <t>template_laudo_fito_v1</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ficha_subcontratacao_als</t>
+          <t>laudo_fito</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>validation_errors</t>
+          <t>classification_audit</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E66" t="b">
         <v>1</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Erros de validacao da saida.</t>
+          <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_bioagri_v1</t>
+          <t>template_laudo_fito_v1</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ficha_recebimento_bioagri</t>
+          <t>laudo_fito</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>results_extract</t>
+          <t>validation_errors</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="E67" t="b">
         <v>1</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Resultados extraidos do PDF para o template.</t>
+          <t>Erros de validacao da saida.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_bioagri_v1</t>
+          <t>template_laudo_mps_v1</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ficha_recebimento_bioagri</t>
+          <t>laudo_mps</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E68" t="b">
         <v>1</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_bioagri_v1</t>
+          <t>template_laudo_mps_v1</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ficha_recebimento_bioagri</t>
+          <t>laudo_mps</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E69" t="b">
         <v>1</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_bioagri_v1</t>
+          <t>template_laudo_mps_v1</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ficha_recebimento_bioagri</t>
+          <t>laudo_mps</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>client</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>98</v>
+        <v>3</v>
       </c>
       <c r="E70" t="b">
         <v>1</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Dados de identificacao do cliente.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>template_ficha_recebimento_bioagri_v1</t>
+          <t>template_laudo_mps_v1</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ficha_recebimento_bioagri</t>
+          <t>laudo_mps</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
+          <t>table_extraction_audit</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>97</v>
+      </c>
+      <c r="E71" t="b">
+        <v>1</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>laudo_mps</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>98</v>
+      </c>
+      <c r="E72" t="b">
+        <v>1</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>template_laudo_mps_v1</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>laudo_mps</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
           <t>validation_errors</t>
         </is>
       </c>
-      <c r="D71" t="n">
+      <c r="D73" t="n">
         <v>99</v>
       </c>
-      <c r="E71" t="b">
-        <v>1</v>
-      </c>
-      <c r="F71" t="inlineStr">
+      <c r="E73" t="b">
+        <v>1</v>
+      </c>
+      <c r="F73" t="inlineStr">
         <is>
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>laudo_sedimento</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" t="b">
+        <v>1</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Resultados extraidos do PDF para o template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>laudo_sedimento</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>2</v>
+      </c>
+      <c r="E75" t="b">
+        <v>1</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Dados de amostra/cabecalho do PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>laudo_sedimento</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>3</v>
+      </c>
+      <c r="E76" t="b">
+        <v>1</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>laudo_sedimento</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>table_extraction_audit</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>97</v>
+      </c>
+      <c r="E77" t="b">
+        <v>1</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>laudo_sedimento</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>98</v>
+      </c>
+      <c r="E78" t="b">
+        <v>1</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>template_laudo_sedimento_v1</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>laudo_sedimento</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>validation_errors</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>99</v>
+      </c>
+      <c r="E79" t="b">
+        <v>1</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Erros de validacao da saida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>laudo_zbt</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" t="b">
+        <v>1</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Resultados extraidos do PDF para o template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>laudo_zbt</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>2</v>
+      </c>
+      <c r="E81" t="b">
+        <v>1</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Dados de amostra/cabecalho do PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>laudo_zbt</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>3</v>
+      </c>
+      <c r="E82" t="b">
+        <v>1</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>laudo_zbt</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>table_extraction_audit</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>97</v>
+      </c>
+      <c r="E83" t="b">
+        <v>1</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>laudo_zbt</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>98</v>
+      </c>
+      <c r="E84" t="b">
+        <v>1</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>template_laudo_zbt_v1</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>laudo_zbt</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>validation_errors</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>99</v>
+      </c>
+      <c r="E85" t="b">
+        <v>1</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Erros de validacao da saida.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F71"/>
+  <autoFilter ref="A1:F85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>